<commit_message>
calibration transparent and pre validation
</commit_message>
<xml_diff>
--- a/scenarios/aim1_results_tables.xlsx
+++ b/scenarios/aim1_results_tables.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="128">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="125">
   <si>
     <t xml:space="preserve">Table 1. Cumulative deaths averted in Indonesia (2025-2050) by intervention scenario.</t>
   </si>
@@ -31,19 +31,19 @@
     <t xml:space="preserve">Antihypertensive Therapy</t>
   </si>
   <si>
-    <t xml:space="preserve">5,312.2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">212.5</t>
+    <t xml:space="preserve">3,570.6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">142.8</t>
   </si>
   <si>
     <t xml:space="preserve">Sodium Reduction</t>
   </si>
   <si>
-    <t xml:space="preserve">2,281.4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">91.3</t>
+    <t xml:space="preserve">1,500.3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">60.0</t>
   </si>
   <si>
     <t xml:space="preserve">Trans-Fat Elimination</t>
@@ -55,19 +55,19 @@
     <t xml:space="preserve">Statin Therapy</t>
   </si>
   <si>
-    <t xml:space="preserve">547.4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">21.9</t>
+    <t xml:space="preserve">392.4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">15.7</t>
   </si>
   <si>
     <t xml:space="preserve">All Interventions</t>
   </si>
   <si>
-    <t xml:space="preserve">7,401.2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">296.0</t>
+    <t xml:space="preserve">4,963.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">198.5</t>
   </si>
   <si>
     <t xml:space="preserve">Table 2. Deaths averted (thousands) by intervention and cause of death.</t>
@@ -94,73 +94,67 @@
     <t xml:space="preserve">Rheumatic heart disease</t>
   </si>
   <si>
-    <t xml:space="preserve">-7.4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">345.6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2,782.1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1,076.6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1,115.4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.1</t>
+    <t xml:space="preserve">-2.3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">248.9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1,737.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">767.6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">818.9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-1.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">74.6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1,035.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">184.7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">207.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">–</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-1.3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-5.9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">351.9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">47.9</t>
   </si>
   <si>
     <t xml:space="preserve">-3.3</t>
   </si>
   <si>
-    <t xml:space="preserve">101.9</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1,652.9</t>
-  </si>
-  <si>
-    <t xml:space="preserve">264.5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">265.7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">–</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-2.4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-13.1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">499.0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">64.7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-10.5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">427.5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3,863.5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1,742.5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1,378.3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.2</t>
+    <t xml:space="preserve">307.8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2,412.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1,230.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1,016.9</t>
   </si>
   <si>
     <t xml:space="preserve">Table 3. Deaths averted by age group and intervention.</t>
@@ -187,31 +181,31 @@
     <t xml:space="preserve">&lt;70</t>
   </si>
   <si>
-    <t xml:space="preserve">11,580,233</t>
-  </si>
-  <si>
-    <t xml:space="preserve">14,183,914</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2,603,682</t>
-  </si>
-  <si>
-    <t xml:space="preserve">104,147</t>
-  </si>
-  <si>
-    <t xml:space="preserve">18.4%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">12,902,181</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1,281,734</t>
-  </si>
-  <si>
-    <t xml:space="preserve">51,269</t>
-  </si>
-  <si>
-    <t xml:space="preserve">9.0%</t>
+    <t xml:space="preserve">7,443,360</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9,017,356</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1,573,996</t>
+  </si>
+  <si>
+    <t xml:space="preserve">62,960</t>
+  </si>
+  <si>
+    <t xml:space="preserve">17.5%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8,260,621</t>
+  </si>
+  <si>
+    <t xml:space="preserve">756,736</t>
+  </si>
+  <si>
+    <t xml:space="preserve">30,269</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8.4%</t>
   </si>
   <si>
     <t xml:space="preserve">0</t>
@@ -220,181 +214,178 @@
     <t xml:space="preserve">0.0%</t>
   </si>
   <si>
-    <t xml:space="preserve">13,925,400</t>
-  </si>
-  <si>
-    <t xml:space="preserve">258,514</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10,341</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.8%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10,492,450</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3,691,464</t>
-  </si>
-  <si>
-    <t xml:space="preserve">147,659</t>
-  </si>
-  <si>
-    <t xml:space="preserve">26.0%</t>
+    <t xml:space="preserve">8,846,992</t>
+  </si>
+  <si>
+    <t xml:space="preserve">170,365</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6,815</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.9%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6,783,960</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2,233,397</t>
+  </si>
+  <si>
+    <t xml:space="preserve">89,336</t>
+  </si>
+  <si>
+    <t xml:space="preserve">24.8%</t>
   </si>
   <si>
     <t xml:space="preserve">70-79</t>
   </si>
   <si>
-    <t xml:space="preserve">6,573,940</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7,810,577</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1,236,638</t>
-  </si>
-  <si>
-    <t xml:space="preserve">49,466</t>
-  </si>
-  <si>
-    <t xml:space="preserve">15.8%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7,398,910</t>
-  </si>
-  <si>
-    <t xml:space="preserve">411,668</t>
-  </si>
-  <si>
-    <t xml:space="preserve">16,467</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5.3%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7,667,537</t>
-  </si>
-  <si>
-    <t xml:space="preserve">143,040</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5,722</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6,118,105</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1,692,472</t>
-  </si>
-  <si>
-    <t xml:space="preserve">67,699</t>
-  </si>
-  <si>
-    <t xml:space="preserve">21.7%</t>
+    <t xml:space="preserve">4,441,035</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5,293,748</t>
+  </si>
+  <si>
+    <t xml:space="preserve">852,714</t>
+  </si>
+  <si>
+    <t xml:space="preserve">34,109</t>
+  </si>
+  <si>
+    <t xml:space="preserve">16.1%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5,018,006</t>
+  </si>
+  <si>
+    <t xml:space="preserve">275,743</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11,030</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.2%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5,190,657</t>
+  </si>
+  <si>
+    <t xml:space="preserve">103,091</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4,124</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4,138,550</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1,155,198</t>
+  </si>
+  <si>
+    <t xml:space="preserve">46,208</t>
+  </si>
+  <si>
+    <t xml:space="preserve">21.8%</t>
   </si>
   <si>
     <t xml:space="preserve">80-89</t>
   </si>
   <si>
-    <t xml:space="preserve">4,654,219</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5,709,154</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1,054,936</t>
-  </si>
-  <si>
-    <t xml:space="preserve">42,197</t>
-  </si>
-  <si>
-    <t xml:space="preserve">18.5%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5,275,447</t>
-  </si>
-  <si>
-    <t xml:space="preserve">433,708</t>
-  </si>
-  <si>
-    <t xml:space="preserve">17,348</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7.6%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5,607,104</t>
-  </si>
-  <si>
-    <t xml:space="preserve">102,050</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4,082</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4,261,930</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1,447,224</t>
-  </si>
-  <si>
-    <t xml:space="preserve">57,889</t>
-  </si>
-  <si>
-    <t xml:space="preserve">25.3%</t>
+    <t xml:space="preserve">3,736,964</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4,555,171</t>
+  </si>
+  <si>
+    <t xml:space="preserve">818,207</t>
+  </si>
+  <si>
+    <t xml:space="preserve">32,728</t>
+  </si>
+  <si>
+    <t xml:space="preserve">18.0%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4,220,931</t>
+  </si>
+  <si>
+    <t xml:space="preserve">334,240</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13,370</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7.3%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4,468,207</t>
+  </si>
+  <si>
+    <t xml:space="preserve">86,964</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3,479</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3,431,099</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1,124,072</t>
+  </si>
+  <si>
+    <t xml:space="preserve">44,963</t>
+  </si>
+  <si>
+    <t xml:space="preserve">24.7%</t>
   </si>
   <si>
     <t xml:space="preserve">90+</t>
   </si>
   <si>
-    <t xml:space="preserve">1,897,820</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2,314,763</t>
-  </si>
-  <si>
-    <t xml:space="preserve">416,944</t>
-  </si>
-  <si>
-    <t xml:space="preserve">16,678</t>
-  </si>
-  <si>
-    <t xml:space="preserve">18.0%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2,160,428</t>
-  </si>
-  <si>
-    <t xml:space="preserve">154,335</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6,173</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6.7%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2,270,949</t>
-  </si>
-  <si>
-    <t xml:space="preserve">43,815</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1,753</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.9%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1,744,765</t>
-  </si>
-  <si>
-    <t xml:space="preserve">569,998</t>
-  </si>
-  <si>
-    <t xml:space="preserve">22,800</t>
+    <t xml:space="preserve">1,506,314</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1,831,989</t>
+  </si>
+  <si>
+    <t xml:space="preserve">325,676</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13,027</t>
+  </si>
+  <si>
+    <t xml:space="preserve">17.8%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1,698,386</t>
+  </si>
+  <si>
+    <t xml:space="preserve">133,603</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5,344</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1,800,054</t>
+  </si>
+  <si>
+    <t xml:space="preserve">31,936</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1,277</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.7%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1,381,127</t>
+  </si>
+  <si>
+    <t xml:space="preserve">450,863</t>
+  </si>
+  <si>
+    <t xml:space="preserve">18,035</t>
   </si>
   <si>
     <t xml:space="preserve">24.6%</t>
@@ -894,7 +885,7 @@
         <v>30</v>
       </c>
       <c r="G4" t="s">
-        <v>31</v>
+        <v>11</v>
       </c>
     </row>
     <row r="5">
@@ -902,22 +893,22 @@
         <v>7</v>
       </c>
       <c r="B5" t="s">
+        <v>31</v>
+      </c>
+      <c r="C5" t="s">
         <v>32</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
         <v>33</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
         <v>34</v>
       </c>
-      <c r="E5" t="s">
+      <c r="F5" t="s">
         <v>35</v>
       </c>
-      <c r="F5" t="s">
-        <v>36</v>
-      </c>
       <c r="G5" t="s">
-        <v>31</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6">
@@ -925,22 +916,22 @@
         <v>10</v>
       </c>
       <c r="B6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="7">
@@ -948,19 +939,19 @@
         <v>12</v>
       </c>
       <c r="B7" t="s">
+        <v>37</v>
+      </c>
+      <c r="C7" t="s">
         <v>38</v>
       </c>
-      <c r="C7" t="s">
+      <c r="D7" t="s">
         <v>39</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E7" t="s">
         <v>40</v>
       </c>
-      <c r="E7" t="s">
+      <c r="F7" t="s">
         <v>41</v>
-      </c>
-      <c r="F7" t="s">
-        <v>42</v>
       </c>
       <c r="G7" t="s">
         <v>11</v>
@@ -971,22 +962,22 @@
         <v>15</v>
       </c>
       <c r="B8" t="s">
+        <v>42</v>
+      </c>
+      <c r="C8" t="s">
         <v>43</v>
       </c>
-      <c r="C8" t="s">
+      <c r="D8" t="s">
         <v>44</v>
       </c>
-      <c r="D8" t="s">
+      <c r="E8" t="s">
         <v>45</v>
       </c>
-      <c r="E8" t="s">
+      <c r="F8" t="s">
         <v>46</v>
       </c>
-      <c r="F8" t="s">
-        <v>47</v>
-      </c>
       <c r="G8" t="s">
-        <v>48</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -1011,490 +1002,490 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>1</v>
       </c>
       <c r="C3" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="E3" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="F3" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="G3" s="2" t="s">
         <v>53</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B4" t="s">
         <v>4</v>
       </c>
       <c r="C4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D4" t="s">
+        <v>56</v>
+      </c>
+      <c r="E4" t="s">
         <v>57</v>
       </c>
-      <c r="D4" t="s">
+      <c r="F4" t="s">
         <v>58</v>
       </c>
-      <c r="E4" t="s">
+      <c r="G4" t="s">
         <v>59</v>
-      </c>
-      <c r="F4" t="s">
-        <v>60</v>
-      </c>
-      <c r="G4" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B5" t="s">
         <v>7</v>
       </c>
       <c r="C5" t="s">
+        <v>60</v>
+      </c>
+      <c r="D5" t="s">
+        <v>56</v>
+      </c>
+      <c r="E5" t="s">
+        <v>61</v>
+      </c>
+      <c r="F5" t="s">
         <v>62</v>
       </c>
-      <c r="D5" t="s">
-        <v>58</v>
-      </c>
-      <c r="E5" t="s">
+      <c r="G5" t="s">
         <v>63</v>
-      </c>
-      <c r="F5" t="s">
-        <v>64</v>
-      </c>
-      <c r="G5" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B6" t="s">
         <v>10</v>
       </c>
       <c r="C6" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="D6" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="E6" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="F6" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="G6" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B7" t="s">
         <v>12</v>
       </c>
       <c r="C7" t="s">
+        <v>66</v>
+      </c>
+      <c r="D7" t="s">
+        <v>56</v>
+      </c>
+      <c r="E7" t="s">
+        <v>67</v>
+      </c>
+      <c r="F7" t="s">
         <v>68</v>
       </c>
-      <c r="D7" t="s">
-        <v>58</v>
-      </c>
-      <c r="E7" t="s">
+      <c r="G7" t="s">
         <v>69</v>
-      </c>
-      <c r="F7" t="s">
-        <v>70</v>
-      </c>
-      <c r="G7" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B8" t="s">
         <v>15</v>
       </c>
       <c r="C8" t="s">
+        <v>70</v>
+      </c>
+      <c r="D8" t="s">
+        <v>56</v>
+      </c>
+      <c r="E8" t="s">
+        <v>71</v>
+      </c>
+      <c r="F8" t="s">
         <v>72</v>
       </c>
-      <c r="D8" t="s">
-        <v>58</v>
-      </c>
-      <c r="E8" t="s">
+      <c r="G8" t="s">
         <v>73</v>
-      </c>
-      <c r="F8" t="s">
-        <v>74</v>
-      </c>
-      <c r="G8" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B9" t="s">
         <v>4</v>
       </c>
       <c r="C9" t="s">
+        <v>75</v>
+      </c>
+      <c r="D9" t="s">
+        <v>76</v>
+      </c>
+      <c r="E9" t="s">
         <v>77</v>
       </c>
-      <c r="D9" t="s">
+      <c r="F9" t="s">
         <v>78</v>
       </c>
-      <c r="E9" t="s">
+      <c r="G9" t="s">
         <v>79</v>
-      </c>
-      <c r="F9" t="s">
-        <v>80</v>
-      </c>
-      <c r="G9" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B10" t="s">
         <v>7</v>
       </c>
       <c r="C10" t="s">
+        <v>80</v>
+      </c>
+      <c r="D10" t="s">
+        <v>76</v>
+      </c>
+      <c r="E10" t="s">
+        <v>81</v>
+      </c>
+      <c r="F10" t="s">
         <v>82</v>
       </c>
-      <c r="D10" t="s">
-        <v>78</v>
-      </c>
-      <c r="E10" t="s">
+      <c r="G10" t="s">
         <v>83</v>
-      </c>
-      <c r="F10" t="s">
-        <v>84</v>
-      </c>
-      <c r="G10" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B11" t="s">
         <v>10</v>
       </c>
       <c r="C11" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="D11" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="E11" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="F11" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="G11" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B12" t="s">
         <v>12</v>
       </c>
       <c r="C12" t="s">
+        <v>84</v>
+      </c>
+      <c r="D12" t="s">
+        <v>76</v>
+      </c>
+      <c r="E12" t="s">
+        <v>85</v>
+      </c>
+      <c r="F12" t="s">
         <v>86</v>
       </c>
-      <c r="D12" t="s">
-        <v>78</v>
-      </c>
-      <c r="E12" t="s">
-        <v>87</v>
-      </c>
-      <c r="F12" t="s">
-        <v>88</v>
-      </c>
       <c r="G12" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B13" t="s">
         <v>15</v>
       </c>
       <c r="C13" t="s">
+        <v>87</v>
+      </c>
+      <c r="D13" t="s">
+        <v>76</v>
+      </c>
+      <c r="E13" t="s">
+        <v>88</v>
+      </c>
+      <c r="F13" t="s">
         <v>89</v>
       </c>
-      <c r="D13" t="s">
-        <v>78</v>
-      </c>
-      <c r="E13" t="s">
+      <c r="G13" t="s">
         <v>90</v>
-      </c>
-      <c r="F13" t="s">
-        <v>91</v>
-      </c>
-      <c r="G13" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B14" t="s">
         <v>4</v>
       </c>
       <c r="C14" t="s">
+        <v>92</v>
+      </c>
+      <c r="D14" t="s">
+        <v>93</v>
+      </c>
+      <c r="E14" t="s">
         <v>94</v>
       </c>
-      <c r="D14" t="s">
+      <c r="F14" t="s">
         <v>95</v>
       </c>
-      <c r="E14" t="s">
+      <c r="G14" t="s">
         <v>96</v>
-      </c>
-      <c r="F14" t="s">
-        <v>97</v>
-      </c>
-      <c r="G14" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B15" t="s">
         <v>7</v>
       </c>
       <c r="C15" t="s">
+        <v>97</v>
+      </c>
+      <c r="D15" t="s">
+        <v>93</v>
+      </c>
+      <c r="E15" t="s">
+        <v>98</v>
+      </c>
+      <c r="F15" t="s">
         <v>99</v>
       </c>
-      <c r="D15" t="s">
-        <v>95</v>
-      </c>
-      <c r="E15" t="s">
+      <c r="G15" t="s">
         <v>100</v>
-      </c>
-      <c r="F15" t="s">
-        <v>101</v>
-      </c>
-      <c r="G15" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B16" t="s">
         <v>10</v>
       </c>
       <c r="C16" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="D16" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="E16" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="F16" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="G16" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B17" t="s">
         <v>12</v>
       </c>
       <c r="C17" t="s">
+        <v>101</v>
+      </c>
+      <c r="D17" t="s">
+        <v>93</v>
+      </c>
+      <c r="E17" t="s">
+        <v>102</v>
+      </c>
+      <c r="F17" t="s">
         <v>103</v>
       </c>
-      <c r="D17" t="s">
-        <v>95</v>
-      </c>
-      <c r="E17" t="s">
-        <v>104</v>
-      </c>
-      <c r="F17" t="s">
-        <v>105</v>
-      </c>
       <c r="G17" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B18" t="s">
         <v>15</v>
       </c>
       <c r="C18" t="s">
+        <v>104</v>
+      </c>
+      <c r="D18" t="s">
+        <v>93</v>
+      </c>
+      <c r="E18" t="s">
+        <v>105</v>
+      </c>
+      <c r="F18" t="s">
         <v>106</v>
       </c>
-      <c r="D18" t="s">
-        <v>95</v>
-      </c>
-      <c r="E18" t="s">
+      <c r="G18" t="s">
         <v>107</v>
-      </c>
-      <c r="F18" t="s">
-        <v>108</v>
-      </c>
-      <c r="G18" t="s">
-        <v>109</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B19" t="s">
         <v>4</v>
       </c>
       <c r="C19" t="s">
+        <v>109</v>
+      </c>
+      <c r="D19" t="s">
+        <v>110</v>
+      </c>
+      <c r="E19" t="s">
         <v>111</v>
       </c>
-      <c r="D19" t="s">
+      <c r="F19" t="s">
         <v>112</v>
       </c>
-      <c r="E19" t="s">
+      <c r="G19" t="s">
         <v>113</v>
-      </c>
-      <c r="F19" t="s">
-        <v>114</v>
-      </c>
-      <c r="G19" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B20" t="s">
         <v>7</v>
       </c>
       <c r="C20" t="s">
+        <v>114</v>
+      </c>
+      <c r="D20" t="s">
+        <v>110</v>
+      </c>
+      <c r="E20" t="s">
+        <v>115</v>
+      </c>
+      <c r="F20" t="s">
         <v>116</v>
       </c>
-      <c r="D20" t="s">
-        <v>112</v>
-      </c>
-      <c r="E20" t="s">
-        <v>117</v>
-      </c>
-      <c r="F20" t="s">
-        <v>118</v>
-      </c>
       <c r="G20" t="s">
-        <v>119</v>
+        <v>100</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B21" t="s">
         <v>10</v>
       </c>
       <c r="C21" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="D21" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E21" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="F21" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="G21" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B22" t="s">
         <v>12</v>
       </c>
       <c r="C22" t="s">
+        <v>117</v>
+      </c>
+      <c r="D22" t="s">
+        <v>110</v>
+      </c>
+      <c r="E22" t="s">
+        <v>118</v>
+      </c>
+      <c r="F22" t="s">
+        <v>119</v>
+      </c>
+      <c r="G22" t="s">
         <v>120</v>
-      </c>
-      <c r="D22" t="s">
-        <v>112</v>
-      </c>
-      <c r="E22" t="s">
-        <v>121</v>
-      </c>
-      <c r="F22" t="s">
-        <v>122</v>
-      </c>
-      <c r="G22" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B23" t="s">
         <v>15</v>
       </c>
       <c r="C23" t="s">
+        <v>121</v>
+      </c>
+      <c r="D23" t="s">
+        <v>110</v>
+      </c>
+      <c r="E23" t="s">
+        <v>122</v>
+      </c>
+      <c r="F23" t="s">
+        <v>123</v>
+      </c>
+      <c r="G23" t="s">
         <v>124</v>
-      </c>
-      <c r="D23" t="s">
-        <v>112</v>
-      </c>
-      <c r="E23" t="s">
-        <v>125</v>
-      </c>
-      <c r="F23" t="s">
-        <v>126</v>
-      </c>
-      <c r="G23" t="s">
-        <v>127</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
calibration transparent by age
</commit_message>
<xml_diff>
--- a/scenarios/aim1_results_tables.xlsx
+++ b/scenarios/aim1_results_tables.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="126">
   <si>
     <t xml:space="preserve">Table 1. Cumulative deaths averted in Indonesia (2025-2050) by intervention scenario.</t>
   </si>
@@ -31,19 +31,19 @@
     <t xml:space="preserve">Antihypertensive Therapy</t>
   </si>
   <si>
-    <t xml:space="preserve">3,570.6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">142.8</t>
+    <t xml:space="preserve">4,687.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">187.5</t>
   </si>
   <si>
     <t xml:space="preserve">Sodium Reduction</t>
   </si>
   <si>
-    <t xml:space="preserve">1,500.3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">60.0</t>
+    <t xml:space="preserve">2,049.9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">82.0</t>
   </si>
   <si>
     <t xml:space="preserve">Trans-Fat Elimination</t>
@@ -55,19 +55,19 @@
     <t xml:space="preserve">Statin Therapy</t>
   </si>
   <si>
-    <t xml:space="preserve">392.4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">15.7</t>
+    <t xml:space="preserve">554.4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">22.2</t>
   </si>
   <si>
     <t xml:space="preserve">All Interventions</t>
   </si>
   <si>
-    <t xml:space="preserve">4,963.5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">198.5</t>
+    <t xml:space="preserve">6,623.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">264.9</t>
   </si>
   <si>
     <t xml:space="preserve">Table 2. Deaths averted (thousands) by intervention and cause of death.</t>
@@ -94,69 +94,72 @@
     <t xml:space="preserve">Rheumatic heart disease</t>
   </si>
   <si>
-    <t xml:space="preserve">-2.3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">248.9</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1,737.5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">767.6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">818.9</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-1.0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">74.6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1,035.1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">184.7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">207.0</t>
+    <t xml:space="preserve">-3.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">288.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2,335.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1,075.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">992.6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-1.6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">86.4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1,444.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">277.3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">243.9</t>
   </si>
   <si>
     <t xml:space="preserve">–</t>
   </si>
   <si>
-    <t xml:space="preserve">-0.2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-1.3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-5.9</t>
-  </si>
-  <si>
-    <t xml:space="preserve">351.9</t>
-  </si>
-  <si>
-    <t xml:space="preserve">47.9</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-3.3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">307.8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2,412.0</t>
+    <t xml:space="preserve">-0.4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-1.9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-9.9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">508.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">58.4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-5.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">357.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3,280.6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1,760.1</t>
   </si>
   <si>
     <t xml:space="preserve">1,230.1</t>
   </si>
   <si>
-    <t xml:space="preserve">1,016.9</t>
-  </si>
-  <si>
     <t xml:space="preserve">Table 3. Deaths averted by age group and intervention.</t>
   </si>
   <si>
@@ -181,31 +184,31 @@
     <t xml:space="preserve">&lt;70</t>
   </si>
   <si>
-    <t xml:space="preserve">7,443,360</t>
-  </si>
-  <si>
-    <t xml:space="preserve">9,017,356</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1,573,996</t>
-  </si>
-  <si>
-    <t xml:space="preserve">62,960</t>
-  </si>
-  <si>
-    <t xml:space="preserve">17.5%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8,260,621</t>
-  </si>
-  <si>
-    <t xml:space="preserve">756,736</t>
-  </si>
-  <si>
-    <t xml:space="preserve">30,269</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8.4%</t>
+    <t xml:space="preserve">12,250,249</t>
+  </si>
+  <si>
+    <t xml:space="preserve">14,824,002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2,573,753</t>
+  </si>
+  <si>
+    <t xml:space="preserve">102,950</t>
+  </si>
+  <si>
+    <t xml:space="preserve">17.4%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13,566,517</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1,257,485</t>
+  </si>
+  <si>
+    <t xml:space="preserve">50,299</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8.5%</t>
   </si>
   <si>
     <t xml:space="preserve">0</t>
@@ -214,181 +217,181 @@
     <t xml:space="preserve">0.0%</t>
   </si>
   <si>
-    <t xml:space="preserve">8,846,992</t>
-  </si>
-  <si>
-    <t xml:space="preserve">170,365</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6,815</t>
+    <t xml:space="preserve">14,516,600</t>
+  </si>
+  <si>
+    <t xml:space="preserve">307,402</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12,296</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.1%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11,124,502</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3,699,500</t>
+  </si>
+  <si>
+    <t xml:space="preserve">147,980</t>
+  </si>
+  <si>
+    <t xml:space="preserve">25.0%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">70-79</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5,673,663</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6,652,220</t>
+  </si>
+  <si>
+    <t xml:space="preserve">978,557</t>
+  </si>
+  <si>
+    <t xml:space="preserve">39,142</t>
+  </si>
+  <si>
+    <t xml:space="preserve">14.7%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6,319,681</t>
+  </si>
+  <si>
+    <t xml:space="preserve">332,539</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13,302</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.0%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6,529,937</t>
+  </si>
+  <si>
+    <t xml:space="preserve">122,282</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4,891</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.8%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5,295,473</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1,356,746</t>
+  </si>
+  <si>
+    <t xml:space="preserve">54,270</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20.4%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">80-89</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3,828,103</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4,634,701</t>
+  </si>
+  <si>
+    <t xml:space="preserve">806,597</t>
+  </si>
+  <si>
+    <t xml:space="preserve">32,264</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4,300,892</t>
+  </si>
+  <si>
+    <t xml:space="preserve">333,808</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13,352</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7.2%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4,548,731</t>
+  </si>
+  <si>
+    <t xml:space="preserve">85,970</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3,439</t>
   </si>
   <si>
     <t xml:space="preserve">1.9%</t>
   </si>
   <si>
-    <t xml:space="preserve">6,783,960</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2,233,397</t>
-  </si>
-  <si>
-    <t xml:space="preserve">89,336</t>
-  </si>
-  <si>
-    <t xml:space="preserve">24.8%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">70-79</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4,441,035</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5,293,748</t>
-  </si>
-  <si>
-    <t xml:space="preserve">852,714</t>
-  </si>
-  <si>
-    <t xml:space="preserve">34,109</t>
-  </si>
-  <si>
-    <t xml:space="preserve">16.1%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5,018,006</t>
-  </si>
-  <si>
-    <t xml:space="preserve">275,743</t>
-  </si>
-  <si>
-    <t xml:space="preserve">11,030</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5.2%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5,190,657</t>
-  </si>
-  <si>
-    <t xml:space="preserve">103,091</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4,124</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4,138,550</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1,155,198</t>
-  </si>
-  <si>
-    <t xml:space="preserve">46,208</t>
-  </si>
-  <si>
-    <t xml:space="preserve">21.8%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">80-89</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3,736,964</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4,555,171</t>
-  </si>
-  <si>
-    <t xml:space="preserve">818,207</t>
-  </si>
-  <si>
-    <t xml:space="preserve">32,728</t>
-  </si>
-  <si>
-    <t xml:space="preserve">18.0%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4,220,931</t>
-  </si>
-  <si>
-    <t xml:space="preserve">334,240</t>
-  </si>
-  <si>
-    <t xml:space="preserve">13,370</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7.3%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4,468,207</t>
-  </si>
-  <si>
-    <t xml:space="preserve">86,964</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3,479</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3,431,099</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1,124,072</t>
-  </si>
-  <si>
-    <t xml:space="preserve">44,963</t>
-  </si>
-  <si>
-    <t xml:space="preserve">24.7%</t>
+    <t xml:space="preserve">3,520,168</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1,114,532</t>
+  </si>
+  <si>
+    <t xml:space="preserve">44,581</t>
+  </si>
+  <si>
+    <t xml:space="preserve">24.0%</t>
   </si>
   <si>
     <t xml:space="preserve">90+</t>
   </si>
   <si>
-    <t xml:space="preserve">1,506,314</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1,831,989</t>
-  </si>
-  <si>
-    <t xml:space="preserve">325,676</t>
-  </si>
-  <si>
-    <t xml:space="preserve">13,027</t>
-  </si>
-  <si>
-    <t xml:space="preserve">17.8%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1,698,386</t>
-  </si>
-  <si>
-    <t xml:space="preserve">133,603</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5,344</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1,800,054</t>
-  </si>
-  <si>
-    <t xml:space="preserve">31,936</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1,277</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.7%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1,381,127</t>
-  </si>
-  <si>
-    <t xml:space="preserve">450,863</t>
-  </si>
-  <si>
-    <t xml:space="preserve">18,035</t>
-  </si>
-  <si>
-    <t xml:space="preserve">24.6%</t>
+    <t xml:space="preserve">1,482,282</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1,810,840</t>
+  </si>
+  <si>
+    <t xml:space="preserve">328,558</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13,142</t>
+  </si>
+  <si>
+    <t xml:space="preserve">18.1%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1,684,771</t>
+  </si>
+  <si>
+    <t xml:space="preserve">126,069</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5,043</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7.0%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1,772,105</t>
+  </si>
+  <si>
+    <t xml:space="preserve">38,736</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1,549</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1,358,428</t>
+  </si>
+  <si>
+    <t xml:space="preserve">452,412</t>
+  </si>
+  <si>
+    <t xml:space="preserve">18,096</t>
   </si>
 </sst>
 </file>
@@ -885,7 +888,7 @@
         <v>30</v>
       </c>
       <c r="G4" t="s">
-        <v>11</v>
+        <v>31</v>
       </c>
     </row>
     <row r="5">
@@ -893,19 +896,19 @@
         <v>7</v>
       </c>
       <c r="B5" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C5" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D5" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F5" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="G5" t="s">
         <v>11</v>
@@ -916,22 +919,22 @@
         <v>10</v>
       </c>
       <c r="B6" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C6" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D6" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E6" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F6" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G6" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="7">
@@ -939,19 +942,19 @@
         <v>12</v>
       </c>
       <c r="B7" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C7" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D7" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E7" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="F7" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G7" t="s">
         <v>11</v>
@@ -962,22 +965,22 @@
         <v>15</v>
       </c>
       <c r="B8" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C8" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D8" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E8" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F8" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G8" t="s">
-        <v>11</v>
+        <v>31</v>
       </c>
     </row>
   </sheetData>
@@ -1002,490 +1005,490 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>1</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B4" t="s">
         <v>4</v>
       </c>
       <c r="C4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D4" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="F4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="G4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B5" t="s">
         <v>7</v>
       </c>
       <c r="C5" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D5" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E5" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="F5" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="G5" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B6" t="s">
         <v>10</v>
       </c>
       <c r="C6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E6" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F6" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="G6" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B7" t="s">
         <v>12</v>
       </c>
       <c r="C7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D7" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E7" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F7" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="G7" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B8" t="s">
         <v>15</v>
       </c>
       <c r="C8" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D8" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E8" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="F8" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="G8" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B9" t="s">
         <v>4</v>
       </c>
       <c r="C9" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D9" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E9" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="F9" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="G9" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B10" t="s">
         <v>7</v>
       </c>
       <c r="C10" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D10" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E10" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F10" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="G10" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B11" t="s">
         <v>10</v>
       </c>
       <c r="C11" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D11" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E11" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F11" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="G11" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B12" t="s">
         <v>12</v>
       </c>
       <c r="C12" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D12" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E12" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="F12" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="G12" t="s">
-        <v>69</v>
+        <v>88</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B13" t="s">
         <v>15</v>
       </c>
       <c r="C13" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D13" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E13" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="F13" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="G13" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B14" t="s">
         <v>4</v>
       </c>
       <c r="C14" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="D14" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="E14" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="F14" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="G14" t="s">
-        <v>96</v>
+        <v>60</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B15" t="s">
         <v>7</v>
       </c>
       <c r="C15" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D15" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="E15" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="F15" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="G15" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B16" t="s">
         <v>10</v>
       </c>
       <c r="C16" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D16" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="E16" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F16" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="G16" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B17" t="s">
         <v>12</v>
       </c>
       <c r="C17" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D17" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="E17" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="F17" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="G17" t="s">
-        <v>69</v>
+        <v>105</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B18" t="s">
         <v>15</v>
       </c>
       <c r="C18" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="D18" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="E18" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="F18" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="G18" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B19" t="s">
         <v>4</v>
       </c>
       <c r="C19" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="D19" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E19" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="F19" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G19" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B20" t="s">
         <v>7</v>
       </c>
       <c r="C20" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="D20" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E20" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="F20" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="G20" t="s">
-        <v>100</v>
+        <v>119</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B21" t="s">
         <v>10</v>
       </c>
       <c r="C21" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D21" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E21" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F21" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="G21" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B22" t="s">
         <v>12</v>
       </c>
       <c r="C22" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="D22" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E22" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="F22" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="G22" t="s">
-        <v>120</v>
+        <v>70</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B23" t="s">
         <v>15</v>
       </c>
       <c r="C23" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="D23" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E23" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="F23" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="G23" t="s">
-        <v>124</v>
+        <v>74</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
pre updating Demography module
</commit_message>
<xml_diff>
--- a/scenarios/aim1_results_tables.xlsx
+++ b/scenarios/aim1_results_tables.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="127">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="175">
   <si>
     <t xml:space="preserve">Table 1. Cumulative deaths averted in Indonesia (2025-2050) by intervention scenario.</t>
   </si>
@@ -70,6 +70,24 @@
     <t xml:space="preserve">304.3</t>
   </si>
   <si>
+    <t xml:space="preserve">FAIR-Choices CVD Package</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3,429.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">137.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">All + FAIR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10,424.6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">417.0</t>
+  </si>
+  <si>
     <t xml:space="preserve">Table 2. Deaths averted (thousands) by intervention and cause of death.</t>
   </si>
   <si>
@@ -160,6 +178,36 @@
     <t xml:space="preserve">1,438.7</t>
   </si>
   <si>
+    <t xml:space="preserve">28.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">342.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">296.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2,088.4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">674.4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">23.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">701.8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3,980.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3,744.8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1,974.8</t>
+  </si>
+  <si>
     <t xml:space="preserve">Table 3. Deaths averted by age group and intervention.</t>
   </si>
   <si>
@@ -241,6 +289,30 @@
     <t xml:space="preserve">25.0%</t>
   </si>
   <si>
+    <t xml:space="preserve">14,841,053</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2,464,584</t>
+  </si>
+  <si>
+    <t xml:space="preserve">98,583</t>
+  </si>
+  <si>
+    <t xml:space="preserve">14.2%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10,993,754</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6,311,883</t>
+  </si>
+  <si>
+    <t xml:space="preserve">252,475</t>
+  </si>
+  <si>
+    <t xml:space="preserve">36.5%</t>
+  </si>
+  <si>
     <t xml:space="preserve">70-79</t>
   </si>
   <si>
@@ -292,6 +364,30 @@
     <t xml:space="preserve">20.3%</t>
   </si>
   <si>
+    <t xml:space="preserve">6,557,311</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1,070,545</t>
+  </si>
+  <si>
+    <t xml:space="preserve">42,822</t>
+  </si>
+  <si>
+    <t xml:space="preserve">14.0%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5,192,975</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2,434,881</t>
+  </si>
+  <si>
+    <t xml:space="preserve">97,395</t>
+  </si>
+  <si>
+    <t xml:space="preserve">31.9%</t>
+  </si>
+  <si>
     <t xml:space="preserve">80-89</t>
   </si>
   <si>
@@ -346,6 +442,30 @@
     <t xml:space="preserve">22.7%</t>
   </si>
   <si>
+    <t xml:space="preserve">5,355,247</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-93,549</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-3,742</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-1.8%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4,113,959</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1,147,739</t>
+  </si>
+  <si>
+    <t xml:space="preserve">45,910</t>
+  </si>
+  <si>
+    <t xml:space="preserve">21.8%</t>
+  </si>
+  <si>
     <t xml:space="preserve">90+</t>
   </si>
   <si>
@@ -395,6 +515,30 @@
   </si>
   <si>
     <t xml:space="preserve">23.2%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2,336,648</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-12,105</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-484</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.5%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1,794,486</t>
+  </si>
+  <si>
+    <t xml:space="preserve">530,058</t>
+  </si>
+  <si>
+    <t xml:space="preserve">21,202</t>
+  </si>
+  <si>
+    <t xml:space="preserve">22.8%</t>
   </si>
 </sst>
 </file>
@@ -823,6 +967,28 @@
         <v>17</v>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B9" t="s">
+        <v>19</v>
+      </c>
+      <c r="C9" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>21</v>
+      </c>
+      <c r="B10" t="s">
+        <v>22</v>
+      </c>
+      <c r="C10" t="s">
+        <v>23</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
@@ -845,30 +1011,30 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
     </row>
     <row r="4">
@@ -876,22 +1042,22 @@
         <v>4</v>
       </c>
       <c r="B4" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="C4" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="D4" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="E4" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="F4" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="G4" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
     </row>
     <row r="5">
@@ -899,19 +1065,19 @@
         <v>7</v>
       </c>
       <c r="B5" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="C5" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="D5" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="E5" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="F5" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="G5" t="s">
         <v>11</v>
@@ -922,22 +1088,22 @@
         <v>10</v>
       </c>
       <c r="B6" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="C6" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="D6" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="E6" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="F6" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="G6" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
     </row>
     <row r="7">
@@ -945,19 +1111,19 @@
         <v>12</v>
       </c>
       <c r="B7" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="C7" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="D7" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="E7" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="F7" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="G7" t="s">
         <v>11</v>
@@ -968,22 +1134,68 @@
         <v>15</v>
       </c>
       <c r="B8" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="C8" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="D8" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="E8" t="s">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="F8" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="G8" t="s">
-        <v>31</v>
+        <v>37</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B9" t="s">
+        <v>54</v>
+      </c>
+      <c r="C9" t="s">
+        <v>55</v>
+      </c>
+      <c r="D9" t="s">
+        <v>56</v>
+      </c>
+      <c r="E9" t="s">
+        <v>57</v>
+      </c>
+      <c r="F9" t="s">
+        <v>58</v>
+      </c>
+      <c r="G9" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>21</v>
+      </c>
+      <c r="B10" t="s">
+        <v>59</v>
+      </c>
+      <c r="C10" t="s">
+        <v>60</v>
+      </c>
+      <c r="D10" t="s">
+        <v>61</v>
+      </c>
+      <c r="E10" t="s">
+        <v>62</v>
+      </c>
+      <c r="F10" t="s">
+        <v>63</v>
+      </c>
+      <c r="G10" t="s">
+        <v>37</v>
       </c>
     </row>
   </sheetData>
@@ -1008,490 +1220,674 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>48</v>
+        <v>64</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>49</v>
+        <v>65</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>1</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>50</v>
+        <v>66</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>51</v>
+        <v>67</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>52</v>
+        <v>68</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>53</v>
+        <v>69</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>54</v>
+        <v>70</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>55</v>
+        <v>71</v>
       </c>
       <c r="B4" t="s">
         <v>4</v>
       </c>
       <c r="C4" t="s">
-        <v>56</v>
+        <v>72</v>
       </c>
       <c r="D4" t="s">
-        <v>57</v>
+        <v>73</v>
       </c>
       <c r="E4" t="s">
-        <v>58</v>
+        <v>74</v>
       </c>
       <c r="F4" t="s">
-        <v>59</v>
+        <v>75</v>
       </c>
       <c r="G4" t="s">
-        <v>60</v>
+        <v>76</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>55</v>
+        <v>71</v>
       </c>
       <c r="B5" t="s">
         <v>7</v>
       </c>
       <c r="C5" t="s">
-        <v>61</v>
+        <v>77</v>
       </c>
       <c r="D5" t="s">
-        <v>57</v>
+        <v>73</v>
       </c>
       <c r="E5" t="s">
-        <v>62</v>
+        <v>78</v>
       </c>
       <c r="F5" t="s">
-        <v>63</v>
+        <v>79</v>
       </c>
       <c r="G5" t="s">
-        <v>64</v>
+        <v>80</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>55</v>
+        <v>71</v>
       </c>
       <c r="B6" t="s">
         <v>10</v>
       </c>
       <c r="C6" t="s">
-        <v>57</v>
+        <v>73</v>
       </c>
       <c r="D6" t="s">
-        <v>57</v>
+        <v>73</v>
       </c>
       <c r="E6" t="s">
-        <v>65</v>
+        <v>81</v>
       </c>
       <c r="F6" t="s">
-        <v>65</v>
+        <v>81</v>
       </c>
       <c r="G6" t="s">
-        <v>66</v>
+        <v>82</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>55</v>
+        <v>71</v>
       </c>
       <c r="B7" t="s">
         <v>12</v>
       </c>
       <c r="C7" t="s">
-        <v>67</v>
+        <v>83</v>
       </c>
       <c r="D7" t="s">
-        <v>57</v>
+        <v>73</v>
       </c>
       <c r="E7" t="s">
-        <v>68</v>
+        <v>84</v>
       </c>
       <c r="F7" t="s">
-        <v>69</v>
+        <v>85</v>
       </c>
       <c r="G7" t="s">
-        <v>70</v>
+        <v>86</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>55</v>
+        <v>71</v>
       </c>
       <c r="B8" t="s">
         <v>15</v>
       </c>
       <c r="C8" t="s">
-        <v>71</v>
+        <v>87</v>
       </c>
       <c r="D8" t="s">
-        <v>57</v>
+        <v>73</v>
       </c>
       <c r="E8" t="s">
-        <v>72</v>
+        <v>88</v>
       </c>
       <c r="F8" t="s">
-        <v>73</v>
+        <v>89</v>
       </c>
       <c r="G8" t="s">
-        <v>74</v>
+        <v>90</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="B9" t="s">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="C9" t="s">
-        <v>76</v>
+        <v>91</v>
       </c>
       <c r="D9" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="E9" t="s">
-        <v>78</v>
+        <v>92</v>
       </c>
       <c r="F9" t="s">
-        <v>79</v>
+        <v>93</v>
       </c>
       <c r="G9" t="s">
-        <v>80</v>
+        <v>94</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="B10" t="s">
-        <v>7</v>
+        <v>21</v>
       </c>
       <c r="C10" t="s">
-        <v>81</v>
+        <v>95</v>
       </c>
       <c r="D10" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="E10" t="s">
-        <v>82</v>
+        <v>96</v>
       </c>
       <c r="F10" t="s">
-        <v>83</v>
+        <v>97</v>
       </c>
       <c r="G10" t="s">
-        <v>84</v>
+        <v>98</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>75</v>
+        <v>99</v>
       </c>
       <c r="B11" t="s">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="C11" t="s">
-        <v>77</v>
+        <v>100</v>
       </c>
       <c r="D11" t="s">
-        <v>77</v>
+        <v>101</v>
       </c>
       <c r="E11" t="s">
-        <v>65</v>
+        <v>102</v>
       </c>
       <c r="F11" t="s">
-        <v>65</v>
+        <v>103</v>
       </c>
       <c r="G11" t="s">
-        <v>66</v>
+        <v>104</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>75</v>
+        <v>99</v>
       </c>
       <c r="B12" t="s">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="C12" t="s">
-        <v>85</v>
+        <v>105</v>
       </c>
       <c r="D12" t="s">
-        <v>77</v>
+        <v>101</v>
       </c>
       <c r="E12" t="s">
-        <v>86</v>
+        <v>106</v>
       </c>
       <c r="F12" t="s">
-        <v>87</v>
+        <v>107</v>
       </c>
       <c r="G12" t="s">
-        <v>70</v>
+        <v>108</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>75</v>
+        <v>99</v>
       </c>
       <c r="B13" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="C13" t="s">
-        <v>88</v>
+        <v>101</v>
       </c>
       <c r="D13" t="s">
-        <v>77</v>
+        <v>101</v>
       </c>
       <c r="E13" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="F13" t="s">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="G13" t="s">
-        <v>91</v>
+        <v>82</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>92</v>
+        <v>99</v>
       </c>
       <c r="B14" t="s">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="C14" t="s">
-        <v>93</v>
+        <v>109</v>
       </c>
       <c r="D14" t="s">
-        <v>94</v>
+        <v>101</v>
       </c>
       <c r="E14" t="s">
-        <v>95</v>
+        <v>110</v>
       </c>
       <c r="F14" t="s">
-        <v>96</v>
+        <v>111</v>
       </c>
       <c r="G14" t="s">
-        <v>97</v>
+        <v>86</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>92</v>
+        <v>99</v>
       </c>
       <c r="B15" t="s">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="C15" t="s">
-        <v>98</v>
+        <v>112</v>
       </c>
       <c r="D15" t="s">
-        <v>94</v>
+        <v>101</v>
       </c>
       <c r="E15" t="s">
-        <v>99</v>
+        <v>113</v>
       </c>
       <c r="F15" t="s">
-        <v>100</v>
+        <v>114</v>
       </c>
       <c r="G15" t="s">
-        <v>101</v>
+        <v>115</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>92</v>
+        <v>99</v>
       </c>
       <c r="B16" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="C16" t="s">
-        <v>94</v>
+        <v>116</v>
       </c>
       <c r="D16" t="s">
-        <v>94</v>
+        <v>101</v>
       </c>
       <c r="E16" t="s">
-        <v>65</v>
+        <v>117</v>
       </c>
       <c r="F16" t="s">
-        <v>65</v>
+        <v>118</v>
       </c>
       <c r="G16" t="s">
-        <v>66</v>
+        <v>119</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>92</v>
+        <v>99</v>
       </c>
       <c r="B17" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="C17" t="s">
-        <v>102</v>
+        <v>120</v>
       </c>
       <c r="D17" t="s">
-        <v>94</v>
+        <v>101</v>
       </c>
       <c r="E17" t="s">
-        <v>103</v>
+        <v>121</v>
       </c>
       <c r="F17" t="s">
-        <v>104</v>
+        <v>122</v>
       </c>
       <c r="G17" t="s">
-        <v>105</v>
+        <v>123</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>92</v>
+        <v>124</v>
       </c>
       <c r="B18" t="s">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="C18" t="s">
-        <v>106</v>
+        <v>125</v>
       </c>
       <c r="D18" t="s">
-        <v>94</v>
+        <v>126</v>
       </c>
       <c r="E18" t="s">
-        <v>107</v>
+        <v>127</v>
       </c>
       <c r="F18" t="s">
-        <v>108</v>
+        <v>128</v>
       </c>
       <c r="G18" t="s">
-        <v>109</v>
+        <v>129</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>110</v>
+        <v>124</v>
       </c>
       <c r="B19" t="s">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C19" t="s">
-        <v>111</v>
+        <v>130</v>
       </c>
       <c r="D19" t="s">
-        <v>112</v>
+        <v>126</v>
       </c>
       <c r="E19" t="s">
-        <v>113</v>
+        <v>131</v>
       </c>
       <c r="F19" t="s">
-        <v>114</v>
+        <v>132</v>
       </c>
       <c r="G19" t="s">
-        <v>115</v>
+        <v>133</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>110</v>
+        <v>124</v>
       </c>
       <c r="B20" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C20" t="s">
-        <v>116</v>
+        <v>126</v>
       </c>
       <c r="D20" t="s">
-        <v>112</v>
+        <v>126</v>
       </c>
       <c r="E20" t="s">
-        <v>117</v>
+        <v>81</v>
       </c>
       <c r="F20" t="s">
-        <v>118</v>
+        <v>81</v>
       </c>
       <c r="G20" t="s">
-        <v>119</v>
+        <v>82</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>110</v>
+        <v>124</v>
       </c>
       <c r="B21" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C21" t="s">
-        <v>112</v>
+        <v>134</v>
       </c>
       <c r="D21" t="s">
-        <v>112</v>
+        <v>126</v>
       </c>
       <c r="E21" t="s">
-        <v>65</v>
+        <v>135</v>
       </c>
       <c r="F21" t="s">
-        <v>65</v>
+        <v>136</v>
       </c>
       <c r="G21" t="s">
-        <v>66</v>
+        <v>137</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>110</v>
+        <v>124</v>
       </c>
       <c r="B22" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C22" t="s">
-        <v>120</v>
+        <v>138</v>
       </c>
       <c r="D22" t="s">
-        <v>112</v>
+        <v>126</v>
       </c>
       <c r="E22" t="s">
-        <v>121</v>
+        <v>139</v>
       </c>
       <c r="F22" t="s">
-        <v>122</v>
+        <v>140</v>
       </c>
       <c r="G22" t="s">
-        <v>70</v>
+        <v>141</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>110</v>
+        <v>124</v>
       </c>
       <c r="B23" t="s">
+        <v>18</v>
+      </c>
+      <c r="C23" t="s">
+        <v>142</v>
+      </c>
+      <c r="D23" t="s">
+        <v>126</v>
+      </c>
+      <c r="E23" t="s">
+        <v>143</v>
+      </c>
+      <c r="F23" t="s">
+        <v>144</v>
+      </c>
+      <c r="G23" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="s">
+        <v>124</v>
+      </c>
+      <c r="B24" t="s">
+        <v>21</v>
+      </c>
+      <c r="C24" t="s">
+        <v>146</v>
+      </c>
+      <c r="D24" t="s">
+        <v>126</v>
+      </c>
+      <c r="E24" t="s">
+        <v>147</v>
+      </c>
+      <c r="F24" t="s">
+        <v>148</v>
+      </c>
+      <c r="G24" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="s">
+        <v>150</v>
+      </c>
+      <c r="B25" t="s">
+        <v>4</v>
+      </c>
+      <c r="C25" t="s">
+        <v>151</v>
+      </c>
+      <c r="D25" t="s">
+        <v>152</v>
+      </c>
+      <c r="E25" t="s">
+        <v>153</v>
+      </c>
+      <c r="F25" t="s">
+        <v>154</v>
+      </c>
+      <c r="G25" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="s">
+        <v>150</v>
+      </c>
+      <c r="B26" t="s">
+        <v>7</v>
+      </c>
+      <c r="C26" t="s">
+        <v>156</v>
+      </c>
+      <c r="D26" t="s">
+        <v>152</v>
+      </c>
+      <c r="E26" t="s">
+        <v>157</v>
+      </c>
+      <c r="F26" t="s">
+        <v>158</v>
+      </c>
+      <c r="G26" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="s">
+        <v>150</v>
+      </c>
+      <c r="B27" t="s">
+        <v>10</v>
+      </c>
+      <c r="C27" t="s">
+        <v>152</v>
+      </c>
+      <c r="D27" t="s">
+        <v>152</v>
+      </c>
+      <c r="E27" t="s">
+        <v>81</v>
+      </c>
+      <c r="F27" t="s">
+        <v>81</v>
+      </c>
+      <c r="G27" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="s">
+        <v>150</v>
+      </c>
+      <c r="B28" t="s">
+        <v>12</v>
+      </c>
+      <c r="C28" t="s">
+        <v>160</v>
+      </c>
+      <c r="D28" t="s">
+        <v>152</v>
+      </c>
+      <c r="E28" t="s">
+        <v>161</v>
+      </c>
+      <c r="F28" t="s">
+        <v>162</v>
+      </c>
+      <c r="G28" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="s">
+        <v>150</v>
+      </c>
+      <c r="B29" t="s">
         <v>15</v>
       </c>
-      <c r="C23" t="s">
-        <v>123</v>
-      </c>
-      <c r="D23" t="s">
-        <v>112</v>
-      </c>
-      <c r="E23" t="s">
-        <v>124</v>
-      </c>
-      <c r="F23" t="s">
-        <v>125</v>
-      </c>
-      <c r="G23" t="s">
-        <v>126</v>
+      <c r="C29" t="s">
+        <v>163</v>
+      </c>
+      <c r="D29" t="s">
+        <v>152</v>
+      </c>
+      <c r="E29" t="s">
+        <v>164</v>
+      </c>
+      <c r="F29" t="s">
+        <v>165</v>
+      </c>
+      <c r="G29" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="s">
+        <v>150</v>
+      </c>
+      <c r="B30" t="s">
+        <v>18</v>
+      </c>
+      <c r="C30" t="s">
+        <v>167</v>
+      </c>
+      <c r="D30" t="s">
+        <v>152</v>
+      </c>
+      <c r="E30" t="s">
+        <v>168</v>
+      </c>
+      <c r="F30" t="s">
+        <v>169</v>
+      </c>
+      <c r="G30" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="s">
+        <v>150</v>
+      </c>
+      <c r="B31" t="s">
+        <v>21</v>
+      </c>
+      <c r="C31" t="s">
+        <v>171</v>
+      </c>
+      <c r="D31" t="s">
+        <v>152</v>
+      </c>
+      <c r="E31" t="s">
+        <v>172</v>
+      </c>
+      <c r="F31" t="s">
+        <v>173</v>
+      </c>
+      <c r="G31" t="s">
+        <v>174</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add FAIR CHoices effect sizes
</commit_message>
<xml_diff>
--- a/scenarios/aim1_results_tables.xlsx
+++ b/scenarios/aim1_results_tables.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="175">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="174">
   <si>
     <t xml:space="preserve">Table 1. Cumulative deaths averted in Indonesia (2025-2050) by intervention scenario.</t>
   </si>
@@ -73,19 +73,19 @@
     <t xml:space="preserve">FAIR-Choices CVD Package</t>
   </si>
   <si>
-    <t xml:space="preserve">3,429.5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">137.2</t>
+    <t xml:space="preserve">998.8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">40.0</t>
   </si>
   <si>
     <t xml:space="preserve">All + FAIR</t>
   </si>
   <si>
-    <t xml:space="preserve">10,424.6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">417.0</t>
+    <t xml:space="preserve">8,453.8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">338.2</t>
   </si>
   <si>
     <t xml:space="preserve">Table 2. Deaths averted (thousands) by intervention and cause of death.</t>
@@ -178,34 +178,34 @@
     <t xml:space="preserve">1,438.7</t>
   </si>
   <si>
-    <t xml:space="preserve">28.5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">342.0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">296.1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2,088.4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">674.4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">23.2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">701.8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3,980.2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3,744.8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1,974.8</t>
+    <t xml:space="preserve">29.6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">158.3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-12.4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">771.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">52.3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">24.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">557.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3,736.6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2,653.3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1,482.8</t>
   </si>
   <si>
     <t xml:space="preserve">Table 3. Deaths averted by age group and intervention.</t>
@@ -289,28 +289,28 @@
     <t xml:space="preserve">25.0%</t>
   </si>
   <si>
-    <t xml:space="preserve">14,841,053</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2,464,584</t>
-  </si>
-  <si>
-    <t xml:space="preserve">98,583</t>
-  </si>
-  <si>
-    <t xml:space="preserve">14.2%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10,993,754</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6,311,883</t>
-  </si>
-  <si>
-    <t xml:space="preserve">252,475</t>
-  </si>
-  <si>
-    <t xml:space="preserve">36.5%</t>
+    <t xml:space="preserve">16,607,726</t>
+  </si>
+  <si>
+    <t xml:space="preserve">697,912</t>
+  </si>
+  <si>
+    <t xml:space="preserve">27,916</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4.0%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12,392,882</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4,912,755</t>
+  </si>
+  <si>
+    <t xml:space="preserve">196,510</t>
+  </si>
+  <si>
+    <t xml:space="preserve">28.4%</t>
   </si>
   <si>
     <t xml:space="preserve">70-79</t>
@@ -364,28 +364,25 @@
     <t xml:space="preserve">20.3%</t>
   </si>
   <si>
-    <t xml:space="preserve">6,557,311</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1,070,545</t>
-  </si>
-  <si>
-    <t xml:space="preserve">42,822</t>
-  </si>
-  <si>
-    <t xml:space="preserve">14.0%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5,192,975</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2,434,881</t>
-  </si>
-  <si>
-    <t xml:space="preserve">97,395</t>
-  </si>
-  <si>
-    <t xml:space="preserve">31.9%</t>
+    <t xml:space="preserve">7,325,906</t>
+  </si>
+  <si>
+    <t xml:space="preserve">301,950</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12,078</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5,828,349</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1,799,507</t>
+  </si>
+  <si>
+    <t xml:space="preserve">71,980</t>
+  </si>
+  <si>
+    <t xml:space="preserve">23.6%</t>
   </si>
   <si>
     <t xml:space="preserve">80-89</t>
@@ -442,28 +439,28 @@
     <t xml:space="preserve">22.7%</t>
   </si>
   <si>
-    <t xml:space="preserve">5,355,247</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-93,549</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-3,742</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-1.8%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4,113,959</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1,147,739</t>
-  </si>
-  <si>
-    <t xml:space="preserve">45,910</t>
-  </si>
-  <si>
-    <t xml:space="preserve">21.8%</t>
+    <t xml:space="preserve">5,264,505</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-2,807</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-112</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.1%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4,062,200</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1,199,498</t>
+  </si>
+  <si>
+    <t xml:space="preserve">47,980</t>
+  </si>
+  <si>
+    <t xml:space="preserve">22.8%</t>
   </si>
   <si>
     <t xml:space="preserve">90+</t>
@@ -517,28 +514,28 @@
     <t xml:space="preserve">23.2%</t>
   </si>
   <si>
-    <t xml:space="preserve">2,336,648</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-12,105</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-484</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.5%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1,794,486</t>
-  </si>
-  <si>
-    <t xml:space="preserve">530,058</t>
-  </si>
-  <si>
-    <t xml:space="preserve">21,202</t>
-  </si>
-  <si>
-    <t xml:space="preserve">22.8%</t>
+    <t xml:space="preserve">2,322,774</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1,769</t>
+  </si>
+  <si>
+    <t xml:space="preserve">71</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.1%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1,782,476</t>
+  </si>
+  <si>
+    <t xml:space="preserve">542,068</t>
+  </si>
+  <si>
+    <t xml:space="preserve">21,683</t>
+  </si>
+  <si>
+    <t xml:space="preserve">23.3%</t>
   </si>
 </sst>
 </file>
@@ -1542,7 +1539,7 @@
         <v>118</v>
       </c>
       <c r="G16" t="s">
-        <v>119</v>
+        <v>94</v>
       </c>
     </row>
     <row r="17">
@@ -1553,79 +1550,79 @@
         <v>21</v>
       </c>
       <c r="C17" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D17" t="s">
         <v>101</v>
       </c>
       <c r="E17" t="s">
+        <v>120</v>
+      </c>
+      <c r="F17" t="s">
         <v>121</v>
       </c>
-      <c r="F17" t="s">
+      <c r="G17" t="s">
         <v>122</v>
-      </c>
-      <c r="G17" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B18" t="s">
         <v>4</v>
       </c>
       <c r="C18" t="s">
+        <v>124</v>
+      </c>
+      <c r="D18" t="s">
         <v>125</v>
       </c>
-      <c r="D18" t="s">
+      <c r="E18" t="s">
         <v>126</v>
       </c>
-      <c r="E18" t="s">
+      <c r="F18" t="s">
         <v>127</v>
       </c>
-      <c r="F18" t="s">
+      <c r="G18" t="s">
         <v>128</v>
-      </c>
-      <c r="G18" t="s">
-        <v>129</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B19" t="s">
         <v>7</v>
       </c>
       <c r="C19" t="s">
+        <v>129</v>
+      </c>
+      <c r="D19" t="s">
+        <v>125</v>
+      </c>
+      <c r="E19" t="s">
         <v>130</v>
       </c>
-      <c r="D19" t="s">
-        <v>126</v>
-      </c>
-      <c r="E19" t="s">
+      <c r="F19" t="s">
         <v>131</v>
       </c>
-      <c r="F19" t="s">
+      <c r="G19" t="s">
         <v>132</v>
-      </c>
-      <c r="G19" t="s">
-        <v>133</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B20" t="s">
         <v>10</v>
       </c>
       <c r="C20" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D20" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="E20" t="s">
         <v>81</v>
@@ -1639,154 +1636,154 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B21" t="s">
         <v>12</v>
       </c>
       <c r="C21" t="s">
+        <v>133</v>
+      </c>
+      <c r="D21" t="s">
+        <v>125</v>
+      </c>
+      <c r="E21" t="s">
         <v>134</v>
       </c>
-      <c r="D21" t="s">
-        <v>126</v>
-      </c>
-      <c r="E21" t="s">
+      <c r="F21" t="s">
         <v>135</v>
       </c>
-      <c r="F21" t="s">
+      <c r="G21" t="s">
         <v>136</v>
-      </c>
-      <c r="G21" t="s">
-        <v>137</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B22" t="s">
         <v>15</v>
       </c>
       <c r="C22" t="s">
+        <v>137</v>
+      </c>
+      <c r="D22" t="s">
+        <v>125</v>
+      </c>
+      <c r="E22" t="s">
         <v>138</v>
       </c>
-      <c r="D22" t="s">
-        <v>126</v>
-      </c>
-      <c r="E22" t="s">
+      <c r="F22" t="s">
         <v>139</v>
       </c>
-      <c r="F22" t="s">
+      <c r="G22" t="s">
         <v>140</v>
-      </c>
-      <c r="G22" t="s">
-        <v>141</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B23" t="s">
         <v>18</v>
       </c>
       <c r="C23" t="s">
+        <v>141</v>
+      </c>
+      <c r="D23" t="s">
+        <v>125</v>
+      </c>
+      <c r="E23" t="s">
         <v>142</v>
       </c>
-      <c r="D23" t="s">
-        <v>126</v>
-      </c>
-      <c r="E23" t="s">
+      <c r="F23" t="s">
         <v>143</v>
       </c>
-      <c r="F23" t="s">
+      <c r="G23" t="s">
         <v>144</v>
-      </c>
-      <c r="G23" t="s">
-        <v>145</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B24" t="s">
         <v>21</v>
       </c>
       <c r="C24" t="s">
+        <v>145</v>
+      </c>
+      <c r="D24" t="s">
+        <v>125</v>
+      </c>
+      <c r="E24" t="s">
         <v>146</v>
       </c>
-      <c r="D24" t="s">
-        <v>126</v>
-      </c>
-      <c r="E24" t="s">
+      <c r="F24" t="s">
         <v>147</v>
       </c>
-      <c r="F24" t="s">
+      <c r="G24" t="s">
         <v>148</v>
-      </c>
-      <c r="G24" t="s">
-        <v>149</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B25" t="s">
         <v>4</v>
       </c>
       <c r="C25" t="s">
+        <v>150</v>
+      </c>
+      <c r="D25" t="s">
         <v>151</v>
       </c>
-      <c r="D25" t="s">
+      <c r="E25" t="s">
         <v>152</v>
       </c>
-      <c r="E25" t="s">
+      <c r="F25" t="s">
         <v>153</v>
       </c>
-      <c r="F25" t="s">
+      <c r="G25" t="s">
         <v>154</v>
-      </c>
-      <c r="G25" t="s">
-        <v>155</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B26" t="s">
         <v>7</v>
       </c>
       <c r="C26" t="s">
+        <v>155</v>
+      </c>
+      <c r="D26" t="s">
+        <v>151</v>
+      </c>
+      <c r="E26" t="s">
         <v>156</v>
       </c>
-      <c r="D26" t="s">
-        <v>152</v>
-      </c>
-      <c r="E26" t="s">
+      <c r="F26" t="s">
         <v>157</v>
       </c>
-      <c r="F26" t="s">
+      <c r="G26" t="s">
         <v>158</v>
-      </c>
-      <c r="G26" t="s">
-        <v>159</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B27" t="s">
         <v>10</v>
       </c>
       <c r="C27" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D27" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="E27" t="s">
         <v>81</v>
@@ -1800,22 +1797,22 @@
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B28" t="s">
         <v>12</v>
       </c>
       <c r="C28" t="s">
+        <v>159</v>
+      </c>
+      <c r="D28" t="s">
+        <v>151</v>
+      </c>
+      <c r="E28" t="s">
         <v>160</v>
       </c>
-      <c r="D28" t="s">
-        <v>152</v>
-      </c>
-      <c r="E28" t="s">
+      <c r="F28" t="s">
         <v>161</v>
-      </c>
-      <c r="F28" t="s">
-        <v>162</v>
       </c>
       <c r="G28" t="s">
         <v>86</v>
@@ -1823,71 +1820,71 @@
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B29" t="s">
         <v>15</v>
       </c>
       <c r="C29" t="s">
+        <v>162</v>
+      </c>
+      <c r="D29" t="s">
+        <v>151</v>
+      </c>
+      <c r="E29" t="s">
         <v>163</v>
       </c>
-      <c r="D29" t="s">
-        <v>152</v>
-      </c>
-      <c r="E29" t="s">
+      <c r="F29" t="s">
         <v>164</v>
       </c>
-      <c r="F29" t="s">
+      <c r="G29" t="s">
         <v>165</v>
-      </c>
-      <c r="G29" t="s">
-        <v>166</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B30" t="s">
         <v>18</v>
       </c>
       <c r="C30" t="s">
+        <v>166</v>
+      </c>
+      <c r="D30" t="s">
+        <v>151</v>
+      </c>
+      <c r="E30" t="s">
         <v>167</v>
       </c>
-      <c r="D30" t="s">
-        <v>152</v>
-      </c>
-      <c r="E30" t="s">
+      <c r="F30" t="s">
         <v>168</v>
       </c>
-      <c r="F30" t="s">
+      <c r="G30" t="s">
         <v>169</v>
-      </c>
-      <c r="G30" t="s">
-        <v>170</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B31" t="s">
         <v>21</v>
       </c>
       <c r="C31" t="s">
+        <v>170</v>
+      </c>
+      <c r="D31" t="s">
+        <v>151</v>
+      </c>
+      <c r="E31" t="s">
         <v>171</v>
       </c>
-      <c r="D31" t="s">
-        <v>152</v>
-      </c>
-      <c r="E31" t="s">
+      <c r="F31" t="s">
         <v>172</v>
       </c>
-      <c r="F31" t="s">
+      <c r="G31" t="s">
         <v>173</v>
-      </c>
-      <c r="G31" t="s">
-        <v>174</v>
       </c>
     </row>
   </sheetData>

</xml_diff>